<commit_message>
Updated readmes, Firmware fixes, V2.0 Controller HArdware
</commit_message>
<xml_diff>
--- a/Hardware/Controller/JLC_PCBA_CPL-DALI_EVG_Controller(V0.2).xlsx
+++ b/Hardware/Controller/JLC_PCBA_CPL-DALI_EVG_Controller(V0.2).xlsx
@@ -624,7 +624,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="0" defaultRowHeight="12.75"/>
   <cols>
     <col width="16.796875" customWidth="1" style="28" min="1" max="1"/>
@@ -765,17 +765,17 @@
       </c>
       <c r="B4" s="19" t="inlineStr">
         <is>
-          <t>20.25</t>
+          <t>26.673</t>
         </is>
       </c>
       <c r="C4" s="19" t="inlineStr">
         <is>
-          <t>9.75</t>
+          <t>8.323</t>
         </is>
       </c>
       <c r="D4" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E4" s="19" t="inlineStr">
@@ -849,17 +849,17 @@
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>34.25</t>
+          <t>34.798</t>
         </is>
       </c>
       <c r="C6" s="19" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>18.263</t>
         </is>
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E6" s="19" t="inlineStr">
@@ -891,12 +891,12 @@
       </c>
       <c r="B7" s="19" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C7" s="19" t="inlineStr">
         <is>
-          <t>21.75</t>
+          <t>21.5</t>
         </is>
       </c>
       <c r="D7" s="19" t="inlineStr">
@@ -975,12 +975,12 @@
       </c>
       <c r="B9" s="19" t="inlineStr">
         <is>
-          <t>30.1</t>
+          <t>30.048</t>
         </is>
       </c>
       <c r="C9" s="19" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7.95</t>
         </is>
       </c>
       <c r="D9" s="19" t="inlineStr">
@@ -1017,17 +1017,17 @@
       </c>
       <c r="B10" s="19" t="inlineStr">
         <is>
-          <t>29.1</t>
+          <t>31.473</t>
         </is>
       </c>
       <c r="C10" s="19" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7.876</t>
         </is>
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>225</t>
         </is>
       </c>
       <c r="E10" s="19" t="inlineStr">
@@ -1059,17 +1059,17 @@
       </c>
       <c r="B11" s="19" t="inlineStr">
         <is>
-          <t>32.36</t>
+          <t>32.75</t>
         </is>
       </c>
       <c r="C11" s="19" t="inlineStr">
         <is>
-          <t>20.091</t>
+          <t>19.25</t>
         </is>
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E11" s="19" t="inlineStr">
@@ -1185,12 +1185,12 @@
       </c>
       <c r="B14" s="19" t="inlineStr">
         <is>
-          <t>30.988</t>
+          <t>30</t>
         </is>
       </c>
       <c r="C14" s="19" t="inlineStr">
         <is>
-          <t>18.339</t>
+          <t>19.25</t>
         </is>
       </c>
       <c r="D14" s="19" t="inlineStr">
@@ -1274,7 +1274,7 @@
       </c>
       <c r="C16" s="19" t="inlineStr">
         <is>
-          <t>20.75</t>
+          <t>20.801</t>
         </is>
       </c>
       <c r="D16" s="19" t="inlineStr">
@@ -1284,7 +1284,7 @@
       </c>
       <c r="E16" s="19" t="inlineStr">
         <is>
-          <t>Top</t>
+          <t>Bottom</t>
         </is>
       </c>
       <c r="F16" s="19" t="inlineStr">
@@ -1311,17 +1311,17 @@
       </c>
       <c r="B17" s="19" t="inlineStr">
         <is>
-          <t>28.7</t>
+          <t>17.5</t>
         </is>
       </c>
       <c r="C17" s="19" t="inlineStr">
         <is>
-          <t>11.1</t>
+          <t>14.5</t>
         </is>
       </c>
       <c r="D17" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E17" s="19" t="inlineStr">
@@ -1348,22 +1348,22 @@
     <row r="18">
       <c r="A18" s="25" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="B18" s="19" t="inlineStr">
         <is>
-          <t>41.25</t>
+          <t>14.25</t>
         </is>
       </c>
       <c r="C18" s="19" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>13.5</t>
         </is>
       </c>
       <c r="D18" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E18" s="19" t="inlineStr">
@@ -1378,34 +1378,34 @@
       </c>
       <c r="G18" s="19" t="inlineStr">
         <is>
-          <t>MB10S</t>
+          <t>B5819W SL</t>
         </is>
       </c>
       <c r="H18" s="19" t="inlineStr">
         <is>
-          <t>SOIC245P670X290-4N</t>
+          <t>SOD-123</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="25" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="B19" s="19" t="inlineStr">
         <is>
-          <t>37</t>
+          <t>41.25</t>
         </is>
       </c>
       <c r="C19" s="19" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D19" s="19" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E19" s="19" t="inlineStr">
@@ -1420,34 +1420,34 @@
       </c>
       <c r="G19" s="19" t="inlineStr">
         <is>
-          <t>BAV99</t>
+          <t>MB10S</t>
         </is>
       </c>
       <c r="H19" s="19" t="inlineStr">
         <is>
-          <t>SOT23</t>
+          <t>SOIC245P670X290-4N</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="25" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="B20" s="19" t="inlineStr">
         <is>
-          <t>29.5</t>
+          <t>37</t>
         </is>
       </c>
       <c r="C20" s="19" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D20" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E20" s="19" t="inlineStr">
@@ -1462,29 +1462,29 @@
       </c>
       <c r="G20" s="19" t="inlineStr">
         <is>
-          <t>B5819W SL</t>
+          <t>BAV99</t>
         </is>
       </c>
       <c r="H20" s="19" t="inlineStr">
         <is>
-          <t>SOD-123</t>
+          <t>SOT23</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="25" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="B21" s="19" t="inlineStr">
         <is>
-          <t>26.25</t>
+          <t>12.25</t>
         </is>
       </c>
       <c r="C21" s="19" t="inlineStr">
         <is>
-          <t>13.75</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="D21" s="19" t="inlineStr">
@@ -1504,34 +1504,34 @@
       </c>
       <c r="G21" s="19" t="inlineStr">
         <is>
-          <t>B5819W SL</t>
+          <t>3V6</t>
         </is>
       </c>
       <c r="H21" s="19" t="inlineStr">
         <is>
-          <t>SOD-123</t>
+          <t>SOD-323</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="25" t="inlineStr">
         <is>
-          <t>D9</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="B22" s="19" t="inlineStr">
         <is>
-          <t>24.25</t>
+          <t>24.562</t>
         </is>
       </c>
       <c r="C22" s="19" t="inlineStr">
         <is>
-          <t>13.75</t>
+          <t>15.164</t>
         </is>
       </c>
       <c r="D22" s="19" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E22" s="19" t="inlineStr">
@@ -1558,22 +1558,22 @@
     <row r="23">
       <c r="A23" s="25" t="inlineStr">
         <is>
-          <t>F1</t>
+          <t>D9</t>
         </is>
       </c>
       <c r="B23" s="19" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>19.75</t>
         </is>
       </c>
       <c r="C23" s="19" t="inlineStr">
         <is>
-          <t>10.5</t>
+          <t>18.5</t>
         </is>
       </c>
       <c r="D23" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E23" s="19" t="inlineStr">
@@ -1588,19 +1588,19 @@
       </c>
       <c r="G23" s="19" t="inlineStr">
         <is>
-          <t>500mA</t>
+          <t>B5819W SL</t>
         </is>
       </c>
       <c r="H23" s="19" t="inlineStr">
         <is>
-          <t>1206</t>
+          <t>SOD-123</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="25" t="inlineStr">
         <is>
-          <t>F2</t>
+          <t>F1</t>
         </is>
       </c>
       <c r="B24" s="19" t="inlineStr">
@@ -1610,12 +1610,12 @@
       </c>
       <c r="C24" s="19" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>10.5</t>
         </is>
       </c>
       <c r="D24" s="19" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E24" s="19" t="inlineStr">
@@ -1642,17 +1642,17 @@
     <row r="25">
       <c r="A25" s="25" t="inlineStr">
         <is>
-          <t>FB1</t>
+          <t>F2</t>
         </is>
       </c>
       <c r="B25" s="19" t="inlineStr">
         <is>
-          <t>28</t>
+          <t>45</t>
         </is>
       </c>
       <c r="C25" s="19" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>15</t>
         </is>
       </c>
       <c r="D25" s="19" t="inlineStr">
@@ -1672,34 +1672,34 @@
       </c>
       <c r="G25" s="19" t="inlineStr">
         <is>
-          <t>GZ1608D601TF</t>
+          <t>500mA</t>
         </is>
       </c>
       <c r="H25" s="19" t="inlineStr">
         <is>
-          <t>0603</t>
+          <t>1206</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="25" t="inlineStr">
         <is>
-          <t>IC1</t>
+          <t>FB1</t>
         </is>
       </c>
       <c r="B26" s="19" t="inlineStr">
         <is>
-          <t>35.5</t>
+          <t>26.67</t>
         </is>
       </c>
       <c r="C26" s="19" t="inlineStr">
         <is>
-          <t>20.75</t>
+          <t>17.78</t>
         </is>
       </c>
       <c r="D26" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E26" s="19" t="inlineStr">
@@ -1714,34 +1714,34 @@
       </c>
       <c r="G26" s="19" t="inlineStr">
         <is>
-          <t>LGS5145</t>
+          <t>GZ1608D601TF</t>
         </is>
       </c>
       <c r="H26" s="19" t="inlineStr">
         <is>
-          <t>SOT95P280X110-6N (SOT23-6L)</t>
+          <t>0603</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t>J1</t>
+          <t>IC1</t>
         </is>
       </c>
       <c r="B27" s="19" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>35.5</t>
         </is>
       </c>
       <c r="C27" s="19" t="inlineStr">
         <is>
-          <t>3.948</t>
+          <t>20.75</t>
         </is>
       </c>
       <c r="D27" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E27" s="19" t="inlineStr">
@@ -1751,17 +1751,17 @@
       </c>
       <c r="F27" s="19" t="inlineStr">
         <is>
-          <t>Not Fitted</t>
+          <t>Fitted</t>
         </is>
       </c>
       <c r="G27" s="19" t="inlineStr">
         <is>
-          <t>USB 3.1 C Receptacle</t>
+          <t>LGS5145</t>
         </is>
       </c>
       <c r="H27" s="19" t="inlineStr">
         <is>
-          <t>C165948</t>
+          <t>SOT95P280X110-6N (SOT23-6L)</t>
         </is>
       </c>
     </row>
@@ -1857,12 +1857,12 @@
       </c>
       <c r="B30" s="19" t="inlineStr">
         <is>
-          <t>11.625</t>
+          <t>18.892</t>
         </is>
       </c>
       <c r="C30" s="19" t="inlineStr">
         <is>
-          <t>11.625</t>
+          <t>4.87</t>
         </is>
       </c>
       <c r="D30" s="19" t="inlineStr">
@@ -1882,76 +1882,76 @@
       </c>
       <c r="G30" s="19" t="inlineStr">
         <is>
-          <t>C262302</t>
+          <t>FFC 0.5mm 10Pin 90°</t>
         </is>
       </c>
       <c r="H30" s="19" t="inlineStr">
         <is>
-          <t>CONN-TH-10P_AFC11-S10ICC-00</t>
+          <t>TE_1-1734592-0</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="25" t="inlineStr">
         <is>
-          <t>J5</t>
+          <t>J6</t>
         </is>
       </c>
       <c r="B31" s="19" t="inlineStr">
         <is>
-          <t>12.383</t>
+          <t>50.775</t>
         </is>
       </c>
       <c r="C31" s="19" t="inlineStr">
         <is>
-          <t>11.625</t>
+          <t>6.785</t>
         </is>
       </c>
       <c r="D31" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E31" s="19" t="inlineStr">
         <is>
-          <t>Bottom</t>
+          <t>Top</t>
         </is>
       </c>
       <c r="F31" s="19" t="inlineStr">
         <is>
-          <t>Not Fitted</t>
+          <t>Fitted</t>
         </is>
       </c>
       <c r="G31" s="19" t="inlineStr">
         <is>
-          <t>C262302</t>
+          <t>Terminalblock X2</t>
         </is>
       </c>
       <c r="H31" s="19" t="inlineStr">
         <is>
-          <t>CONN-TH-10P_AFC11-S10ICC-00</t>
+          <t>Terminalblock_X2_5mm</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="25" t="inlineStr">
         <is>
-          <t>L1</t>
+          <t>J7</t>
         </is>
       </c>
       <c r="B32" s="19" t="inlineStr">
         <is>
-          <t>32.741</t>
+          <t>50.775</t>
         </is>
       </c>
       <c r="C32" s="19" t="inlineStr">
         <is>
-          <t>15.418</t>
+          <t>16.945</t>
         </is>
       </c>
       <c r="D32" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E32" s="19" t="inlineStr">
@@ -1966,34 +1966,34 @@
       </c>
       <c r="G32" s="19" t="inlineStr">
         <is>
-          <t>CMI321609X100KT (10uH)</t>
+          <t>Terminalblock X2</t>
         </is>
       </c>
       <c r="H32" s="19" t="inlineStr">
         <is>
-          <t>L1210</t>
+          <t>Terminalblock_X2_5mm</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="25" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>L1</t>
         </is>
       </c>
       <c r="B33" s="19" t="inlineStr">
         <is>
-          <t>29.845</t>
+          <t>32.741</t>
         </is>
       </c>
       <c r="C33" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>15.418</t>
         </is>
       </c>
       <c r="D33" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E33" s="19" t="inlineStr">
@@ -2003,39 +2003,39 @@
       </c>
       <c r="F33" s="19" t="inlineStr">
         <is>
-          <t>Not Fitted</t>
+          <t>Fitted</t>
         </is>
       </c>
       <c r="G33" s="19" t="inlineStr">
         <is>
-          <t>4 Pin male</t>
+          <t>CMI321609X100KT (10uH)</t>
         </is>
       </c>
       <c r="H33" s="19" t="inlineStr">
         <is>
-          <t>TE_826647-4</t>
+          <t>L1210</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="25" t="inlineStr">
         <is>
-          <t>P5</t>
+          <t>P3</t>
         </is>
       </c>
       <c r="B34" s="19" t="inlineStr">
         <is>
-          <t>47.75</t>
+          <t>29.845</t>
         </is>
       </c>
       <c r="C34" s="19" t="inlineStr">
         <is>
-          <t>12.292</t>
+          <t>0</t>
         </is>
       </c>
       <c r="D34" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E34" s="19" t="inlineStr">
@@ -2045,17 +2045,17 @@
       </c>
       <c r="F34" s="19" t="inlineStr">
         <is>
-          <t>Fitted</t>
+          <t>Not Fitted</t>
         </is>
       </c>
       <c r="G34" s="19" t="inlineStr">
         <is>
-          <t>KF2EDGR-3.5-4Pin</t>
+          <t>4 Pin male</t>
         </is>
       </c>
       <c r="H34" s="19" t="inlineStr">
         <is>
-          <t>CONN-TH_4P-P3.50_KF2EDGR-3.5-4P</t>
+          <t>TE_826647-4</t>
         </is>
       </c>
     </row>
@@ -2193,12 +2193,12 @@
       </c>
       <c r="B38" s="19" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>20.25</t>
         </is>
       </c>
       <c r="C38" s="19" t="inlineStr">
         <is>
-          <t>13.75</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="D38" s="19" t="inlineStr">
@@ -2235,17 +2235,17 @@
       </c>
       <c r="B39" s="19" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>19.5</t>
         </is>
       </c>
       <c r="C39" s="19" t="inlineStr">
         <is>
-          <t>18.25</t>
+          <t>11.75</t>
         </is>
       </c>
       <c r="D39" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E39" s="19" t="inlineStr">
@@ -2272,22 +2272,22 @@
     <row r="40">
       <c r="A40" s="25" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="B40" s="19" t="inlineStr">
         <is>
-          <t>20.75</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C40" s="19" t="inlineStr">
         <is>
-          <t>17.5</t>
+          <t>8.5</t>
         </is>
       </c>
       <c r="D40" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E40" s="19" t="inlineStr">
@@ -2302,12 +2302,12 @@
       </c>
       <c r="G40" s="19" t="inlineStr">
         <is>
-          <t>MMBT5551</t>
+          <t>2N7002</t>
         </is>
       </c>
       <c r="H40" s="19" t="inlineStr">
         <is>
-          <t>SOT23 Reverse</t>
+          <t>SOT23 Normal</t>
         </is>
       </c>
     </row>
@@ -2319,17 +2319,17 @@
       </c>
       <c r="B41" s="19" t="inlineStr">
         <is>
-          <t>31</t>
+          <t>15</t>
         </is>
       </c>
       <c r="C41" s="19" t="inlineStr">
         <is>
-          <t>10.5</t>
+          <t>15.5</t>
         </is>
       </c>
       <c r="D41" s="19" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E41" s="19" t="inlineStr">
@@ -2487,17 +2487,17 @@
       </c>
       <c r="B45" s="19" t="inlineStr">
         <is>
-          <t>14.5</t>
+          <t>18.25</t>
         </is>
       </c>
       <c r="C45" s="19" t="inlineStr">
         <is>
-          <t>17.75</t>
+          <t>9.25</t>
         </is>
       </c>
       <c r="D45" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E45" s="19" t="inlineStr">
@@ -2529,17 +2529,17 @@
       </c>
       <c r="B46" s="19" t="inlineStr">
         <is>
-          <t>18.5</t>
+          <t>10.75</t>
         </is>
       </c>
       <c r="C46" s="19" t="inlineStr">
         <is>
-          <t>21.6</t>
+          <t>13.25</t>
         </is>
       </c>
       <c r="D46" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E46" s="19" t="inlineStr">
@@ -2554,7 +2554,7 @@
       </c>
       <c r="G46" s="19" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>33k</t>
         </is>
       </c>
       <c r="H46" s="19" t="inlineStr">
@@ -2566,22 +2566,22 @@
     <row r="47">
       <c r="A47" s="25" t="inlineStr">
         <is>
-          <t>R7</t>
+          <t>R8</t>
         </is>
       </c>
       <c r="B47" s="19" t="inlineStr">
         <is>
-          <t>15.4</t>
+          <t>26.035</t>
         </is>
       </c>
       <c r="C47" s="19" t="inlineStr">
         <is>
-          <t>21.6</t>
+          <t>7.036</t>
         </is>
       </c>
       <c r="D47" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E47" s="19" t="inlineStr">
@@ -2601,29 +2601,29 @@
       </c>
       <c r="H47" s="19" t="inlineStr">
         <is>
-          <t>R0603</t>
+          <t>0402</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="25" t="inlineStr">
         <is>
-          <t>R8</t>
+          <t>R9</t>
         </is>
       </c>
       <c r="B48" s="19" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>26.086</t>
         </is>
       </c>
       <c r="C48" s="19" t="inlineStr">
         <is>
-          <t>9.75</t>
+          <t>5.258</t>
         </is>
       </c>
       <c r="D48" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E48" s="19" t="inlineStr">
@@ -2650,17 +2650,17 @@
     <row r="49">
       <c r="A49" s="25" t="inlineStr">
         <is>
-          <t>R9</t>
+          <t>R10</t>
         </is>
       </c>
       <c r="B49" s="19" t="inlineStr">
         <is>
-          <t>26</t>
+          <t>41.5</t>
         </is>
       </c>
       <c r="C49" s="19" t="inlineStr">
         <is>
-          <t>10.75</t>
+          <t>7.5</t>
         </is>
       </c>
       <c r="D49" s="19" t="inlineStr">
@@ -2680,29 +2680,29 @@
       </c>
       <c r="G49" s="19" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H49" s="19" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>R0603</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="25" t="inlineStr">
         <is>
-          <t>R10</t>
+          <t>R11</t>
         </is>
       </c>
       <c r="B50" s="19" t="inlineStr">
         <is>
-          <t>41.5</t>
+          <t>13.25</t>
         </is>
       </c>
       <c r="C50" s="19" t="inlineStr">
         <is>
-          <t>7.5</t>
+          <t>11.25</t>
         </is>
       </c>
       <c r="D50" s="19" t="inlineStr">
@@ -2722,7 +2722,7 @@
       </c>
       <c r="G50" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>47k</t>
         </is>
       </c>
       <c r="H50" s="19" t="inlineStr">
@@ -2734,22 +2734,22 @@
     <row r="51">
       <c r="A51" s="25" t="inlineStr">
         <is>
-          <t>R11</t>
+          <t>R12</t>
         </is>
       </c>
       <c r="B51" s="19" t="inlineStr">
         <is>
-          <t>14.3</t>
+          <t>32.75</t>
         </is>
       </c>
       <c r="C51" s="19" t="inlineStr">
         <is>
-          <t>20.1</t>
+          <t>21.25</t>
         </is>
       </c>
       <c r="D51" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E51" s="19" t="inlineStr">
@@ -2764,34 +2764,34 @@
       </c>
       <c r="G51" s="19" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>15k</t>
         </is>
       </c>
       <c r="H51" s="19" t="inlineStr">
         <is>
-          <t>R0603</t>
+          <t>0402</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="25" t="inlineStr">
         <is>
-          <t>R12</t>
+          <t>R18</t>
         </is>
       </c>
       <c r="B52" s="19" t="inlineStr">
         <is>
-          <t>39.65</t>
+          <t>6.5</t>
         </is>
       </c>
       <c r="C52" s="19" t="inlineStr">
         <is>
-          <t>22.075</t>
+          <t>19.75</t>
         </is>
       </c>
       <c r="D52" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E52" s="19" t="inlineStr">
@@ -2806,7 +2806,7 @@
       </c>
       <c r="G52" s="19" t="inlineStr">
         <is>
-          <t>15k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="H52" s="19" t="inlineStr">
@@ -2818,7 +2818,7 @@
     <row r="53">
       <c r="A53" s="25" t="inlineStr">
         <is>
-          <t>R18</t>
+          <t>R23</t>
         </is>
       </c>
       <c r="B53" s="19" t="inlineStr">
@@ -2828,7 +2828,7 @@
       </c>
       <c r="C53" s="19" t="inlineStr">
         <is>
-          <t>19.75</t>
+          <t>4.75</t>
         </is>
       </c>
       <c r="D53" s="19" t="inlineStr">
@@ -2860,17 +2860,17 @@
     <row r="54">
       <c r="A54" s="25" t="inlineStr">
         <is>
-          <t>R19</t>
+          <t>R27</t>
         </is>
       </c>
       <c r="B54" s="19" t="inlineStr">
         <is>
-          <t>24.5</t>
+          <t>23.5</t>
         </is>
       </c>
       <c r="C54" s="19" t="inlineStr">
         <is>
-          <t>4.25</t>
+          <t>17.75</t>
         </is>
       </c>
       <c r="D54" s="19" t="inlineStr">
@@ -2890,34 +2890,34 @@
       </c>
       <c r="G54" s="19" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H54" s="19" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>R0603</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="25" t="inlineStr">
         <is>
-          <t>R20</t>
+          <t>R28</t>
         </is>
       </c>
       <c r="B55" s="19" t="inlineStr">
         <is>
-          <t>25.5</t>
+          <t>38.5</t>
         </is>
       </c>
       <c r="C55" s="19" t="inlineStr">
         <is>
-          <t>4.25</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D55" s="19" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>0</t>
         </is>
       </c>
       <c r="E55" s="19" t="inlineStr">
@@ -2932,34 +2932,34 @@
       </c>
       <c r="G55" s="19" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>1M</t>
         </is>
       </c>
       <c r="H55" s="19" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>R0603</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="25" t="inlineStr">
         <is>
-          <t>R21</t>
+          <t>R29</t>
         </is>
       </c>
       <c r="B56" s="19" t="inlineStr">
         <is>
-          <t>23</t>
+          <t>33</t>
         </is>
       </c>
       <c r="C56" s="19" t="inlineStr">
         <is>
-          <t>9.35</t>
+          <t>12.75</t>
         </is>
       </c>
       <c r="D56" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E56" s="19" t="inlineStr">
@@ -2974,29 +2974,29 @@
       </c>
       <c r="G56" s="19" t="inlineStr">
         <is>
-          <t>1.5k</t>
+          <t>1k</t>
         </is>
       </c>
       <c r="H56" s="19" t="inlineStr">
         <is>
-          <t>R0603</t>
+          <t>0402</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="25" t="inlineStr">
         <is>
-          <t>R22</t>
+          <t>R30</t>
         </is>
       </c>
       <c r="B57" s="19" t="inlineStr">
         <is>
-          <t>21.5</t>
+          <t>37.75</t>
         </is>
       </c>
       <c r="C57" s="19" t="inlineStr">
         <is>
-          <t>9.35</t>
+          <t>10.25</t>
         </is>
       </c>
       <c r="D57" s="19" t="inlineStr">
@@ -3011,12 +3011,12 @@
       </c>
       <c r="F57" s="19" t="inlineStr">
         <is>
-          <t>Not Fitted</t>
+          <t>Fitted</t>
         </is>
       </c>
       <c r="G57" s="19" t="inlineStr">
         <is>
-          <t>1.5k</t>
+          <t>4.7k</t>
         </is>
       </c>
       <c r="H57" s="19" t="inlineStr">
@@ -3028,17 +3028,17 @@
     <row r="58">
       <c r="A58" s="25" t="inlineStr">
         <is>
-          <t>R23</t>
+          <t>R31</t>
         </is>
       </c>
       <c r="B58" s="19" t="inlineStr">
         <is>
-          <t>6.5</t>
+          <t>37.25</t>
         </is>
       </c>
       <c r="C58" s="19" t="inlineStr">
         <is>
-          <t>4.75</t>
+          <t>5.75</t>
         </is>
       </c>
       <c r="D58" s="19" t="inlineStr">
@@ -3058,34 +3058,34 @@
       </c>
       <c r="G58" s="19" t="inlineStr">
         <is>
-          <t>10k</t>
+          <t>100k</t>
         </is>
       </c>
       <c r="H58" s="19" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>R0603</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="25" t="inlineStr">
         <is>
-          <t>R27</t>
+          <t>R32</t>
         </is>
       </c>
       <c r="B59" s="19" t="inlineStr">
         <is>
-          <t>23.5</t>
+          <t>37.75</t>
         </is>
       </c>
       <c r="C59" s="19" t="inlineStr">
         <is>
-          <t>17.75</t>
+          <t>13.25</t>
         </is>
       </c>
       <c r="D59" s="19" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E59" s="19" t="inlineStr">
@@ -3100,7 +3100,7 @@
       </c>
       <c r="G59" s="19" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8.2k</t>
         </is>
       </c>
       <c r="H59" s="19" t="inlineStr">
@@ -3112,22 +3112,22 @@
     <row r="60">
       <c r="A60" s="25" t="inlineStr">
         <is>
-          <t>R28</t>
+          <t>R33</t>
         </is>
       </c>
       <c r="B60" s="19" t="inlineStr">
         <is>
-          <t>38.5</t>
+          <t>35.75</t>
         </is>
       </c>
       <c r="C60" s="19" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5.75</t>
         </is>
       </c>
       <c r="D60" s="19" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E60" s="19" t="inlineStr">
@@ -3142,7 +3142,7 @@
       </c>
       <c r="G60" s="19" t="inlineStr">
         <is>
-          <t>1M</t>
+          <t>18k</t>
         </is>
       </c>
       <c r="H60" s="19" t="inlineStr">
@@ -3154,22 +3154,22 @@
     <row r="61">
       <c r="A61" s="25" t="inlineStr">
         <is>
-          <t>R29</t>
+          <t>R41</t>
         </is>
       </c>
       <c r="B61" s="19" t="inlineStr">
         <is>
-          <t>33</t>
+          <t>25</t>
         </is>
       </c>
       <c r="C61" s="19" t="inlineStr">
         <is>
-          <t>12.75</t>
+          <t>18</t>
         </is>
       </c>
       <c r="D61" s="19" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E61" s="19" t="inlineStr">
@@ -3184,34 +3184,34 @@
       </c>
       <c r="G61" s="19" t="inlineStr">
         <is>
-          <t>1k</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H61" s="19" t="inlineStr">
         <is>
-          <t>0402</t>
+          <t>R0603</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="25" t="inlineStr">
         <is>
-          <t>R30</t>
+          <t>R46</t>
         </is>
       </c>
       <c r="B62" s="19" t="inlineStr">
         <is>
-          <t>37.75</t>
+          <t>39.5</t>
         </is>
       </c>
       <c r="C62" s="19" t="inlineStr">
         <is>
-          <t>10.25</t>
+          <t>18.75</t>
         </is>
       </c>
       <c r="D62" s="19" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E62" s="19" t="inlineStr">
@@ -3226,7 +3226,7 @@
       </c>
       <c r="G62" s="19" t="inlineStr">
         <is>
-          <t>4.7k</t>
+          <t>33k</t>
         </is>
       </c>
       <c r="H62" s="19" t="inlineStr">
@@ -3238,22 +3238,22 @@
     <row r="63">
       <c r="A63" s="25" t="inlineStr">
         <is>
-          <t>R31</t>
+          <t>R47</t>
         </is>
       </c>
       <c r="B63" s="19" t="inlineStr">
         <is>
-          <t>37.25</t>
+          <t>38.225</t>
         </is>
       </c>
       <c r="C63" s="19" t="inlineStr">
         <is>
-          <t>5.75</t>
+          <t>20.8</t>
         </is>
       </c>
       <c r="D63" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>270</t>
         </is>
       </c>
       <c r="E63" s="19" t="inlineStr">
@@ -3268,34 +3268,34 @@
       </c>
       <c r="G63" s="19" t="inlineStr">
         <is>
-          <t>100k</t>
+          <t>10k</t>
         </is>
       </c>
       <c r="H63" s="19" t="inlineStr">
         <is>
-          <t>R0603</t>
+          <t>0402</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="25" t="inlineStr">
         <is>
-          <t>R32</t>
+          <t>U1</t>
         </is>
       </c>
       <c r="B64" s="19" t="inlineStr">
         <is>
-          <t>37.75</t>
+          <t>30.261</t>
         </is>
       </c>
       <c r="C64" s="19" t="inlineStr">
         <is>
-          <t>13.25</t>
+          <t>4.671</t>
         </is>
       </c>
       <c r="D64" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>225</t>
         </is>
       </c>
       <c r="E64" s="19" t="inlineStr">
@@ -3310,34 +3310,34 @@
       </c>
       <c r="G64" s="19" t="inlineStr">
         <is>
-          <t>8.2k</t>
+          <t>CH32V003F4U6</t>
         </is>
       </c>
       <c r="H64" s="19" t="inlineStr">
         <is>
-          <t>R0603</t>
+          <t>QFN-20_L3.0-W3.0-P0.40-TL-EP1.7</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="25" t="inlineStr">
         <is>
-          <t>R33</t>
+          <t>U2</t>
         </is>
       </c>
       <c r="B65" s="19" t="inlineStr">
         <is>
-          <t>35.75</t>
+          <t>34.75</t>
         </is>
       </c>
       <c r="C65" s="19" t="inlineStr">
         <is>
-          <t>5.75</t>
+          <t>9.75</t>
         </is>
       </c>
       <c r="D65" s="19" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>90</t>
         </is>
       </c>
       <c r="E65" s="19" t="inlineStr">
@@ -3352,34 +3352,34 @@
       </c>
       <c r="G65" s="19" t="inlineStr">
         <is>
-          <t>18k</t>
+          <t>LMV331IDBVRG4</t>
         </is>
       </c>
       <c r="H65" s="19" t="inlineStr">
         <is>
-          <t>R0603</t>
+          <t>SOT23-5</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="25" t="inlineStr">
         <is>
-          <t>R41</t>
+          <t>U3</t>
         </is>
       </c>
       <c r="B66" s="19" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>26.739</t>
         </is>
       </c>
       <c r="C66" s="19" t="inlineStr">
         <is>
-          <t>17.75</t>
+          <t>11.382</t>
         </is>
       </c>
       <c r="D66" s="19" t="inlineStr">
         <is>
-          <t>90</t>
+          <t>180</t>
         </is>
       </c>
       <c r="E66" s="19" t="inlineStr">
@@ -3394,262 +3394,10 @@
       </c>
       <c r="G66" s="19" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>AT24C256C-SSHL-T</t>
         </is>
       </c>
       <c r="H66" s="19" t="inlineStr">
-        <is>
-          <t>R0603</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="25" t="inlineStr">
-        <is>
-          <t>R42</t>
-        </is>
-      </c>
-      <c r="B67" s="19" t="inlineStr">
-        <is>
-          <t>26.5</t>
-        </is>
-      </c>
-      <c r="C67" s="19" t="inlineStr">
-        <is>
-          <t>17.75</t>
-        </is>
-      </c>
-      <c r="D67" s="19" t="inlineStr">
-        <is>
-          <t>270</t>
-        </is>
-      </c>
-      <c r="E67" s="19" t="inlineStr">
-        <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="F67" s="19" t="inlineStr">
-        <is>
-          <t>Fitted</t>
-        </is>
-      </c>
-      <c r="G67" s="19" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="H67" s="19" t="inlineStr">
-        <is>
-          <t>R0603</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="25" t="inlineStr">
-        <is>
-          <t>R46</t>
-        </is>
-      </c>
-      <c r="B68" s="19" t="inlineStr">
-        <is>
-          <t>39.5</t>
-        </is>
-      </c>
-      <c r="C68" s="19" t="inlineStr">
-        <is>
-          <t>18.75</t>
-        </is>
-      </c>
-      <c r="D68" s="19" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
-      </c>
-      <c r="E68" s="19" t="inlineStr">
-        <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="F68" s="19" t="inlineStr">
-        <is>
-          <t>Fitted</t>
-        </is>
-      </c>
-      <c r="G68" s="19" t="inlineStr">
-        <is>
-          <t>33k</t>
-        </is>
-      </c>
-      <c r="H68" s="19" t="inlineStr">
-        <is>
-          <t>R0603</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" s="25" t="inlineStr">
-        <is>
-          <t>R47</t>
-        </is>
-      </c>
-      <c r="B69" s="19" t="inlineStr">
-        <is>
-          <t>38.225</t>
-        </is>
-      </c>
-      <c r="C69" s="19" t="inlineStr">
-        <is>
-          <t>20.8</t>
-        </is>
-      </c>
-      <c r="D69" s="19" t="inlineStr">
-        <is>
-          <t>270</t>
-        </is>
-      </c>
-      <c r="E69" s="19" t="inlineStr">
-        <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="F69" s="19" t="inlineStr">
-        <is>
-          <t>Fitted</t>
-        </is>
-      </c>
-      <c r="G69" s="19" t="inlineStr">
-        <is>
-          <t>10k</t>
-        </is>
-      </c>
-      <c r="H69" s="19" t="inlineStr">
-        <is>
-          <t>0402</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="25" t="inlineStr">
-        <is>
-          <t>U1</t>
-        </is>
-      </c>
-      <c r="B70" s="19" t="inlineStr">
-        <is>
-          <t>30.261</t>
-        </is>
-      </c>
-      <c r="C70" s="19" t="inlineStr">
-        <is>
-          <t>4.671</t>
-        </is>
-      </c>
-      <c r="D70" s="19" t="inlineStr">
-        <is>
-          <t>225</t>
-        </is>
-      </c>
-      <c r="E70" s="19" t="inlineStr">
-        <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="F70" s="19" t="inlineStr">
-        <is>
-          <t>Fitted</t>
-        </is>
-      </c>
-      <c r="G70" s="19" t="inlineStr">
-        <is>
-          <t>CH32V003F4U6</t>
-        </is>
-      </c>
-      <c r="H70" s="19" t="inlineStr">
-        <is>
-          <t>QFN-20_L3.0-W3.0-P0.40-TL-EP1.7</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="25" t="inlineStr">
-        <is>
-          <t>U2</t>
-        </is>
-      </c>
-      <c r="B71" s="19" t="inlineStr">
-        <is>
-          <t>34.75</t>
-        </is>
-      </c>
-      <c r="C71" s="19" t="inlineStr">
-        <is>
-          <t>9.75</t>
-        </is>
-      </c>
-      <c r="D71" s="19" t="inlineStr">
-        <is>
-          <t>90</t>
-        </is>
-      </c>
-      <c r="E71" s="19" t="inlineStr">
-        <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="F71" s="19" t="inlineStr">
-        <is>
-          <t>Fitted</t>
-        </is>
-      </c>
-      <c r="G71" s="19" t="inlineStr">
-        <is>
-          <t>LMV331IDBVRG4</t>
-        </is>
-      </c>
-      <c r="H71" s="19" t="inlineStr">
-        <is>
-          <t>SOT23-5</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="25" t="inlineStr">
-        <is>
-          <t>U3</t>
-        </is>
-      </c>
-      <c r="B72" s="19" t="inlineStr">
-        <is>
-          <t>17</t>
-        </is>
-      </c>
-      <c r="C72" s="19" t="inlineStr">
-        <is>
-          <t>12</t>
-        </is>
-      </c>
-      <c r="D72" s="19" t="inlineStr">
-        <is>
-          <t>270</t>
-        </is>
-      </c>
-      <c r="E72" s="19" t="inlineStr">
-        <is>
-          <t>Top</t>
-        </is>
-      </c>
-      <c r="F72" s="19" t="inlineStr">
-        <is>
-          <t>Fitted</t>
-        </is>
-      </c>
-      <c r="G72" s="19" t="inlineStr">
-        <is>
-          <t>AT24C256C-SSHL-T</t>
-        </is>
-      </c>
-      <c r="H72" s="19" t="inlineStr">
         <is>
           <t>SOIC127P600X265-8N (SOIC-8)</t>
         </is>

</xml_diff>